<commit_message>
fix: use openpyxl directly for deterministic xlsx generation
Refs: TASK-DELETE.7
</commit_message>
<xml_diff>
--- a/mock_data/mvp2a3_core.xlsx
+++ b/mock_data/mvp2a3_core.xlsx
@@ -734,9 +734,15 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
+      <c r="AF2" t="n">
+        <v/>
+      </c>
+      <c r="AG2" t="n">
+        <v/>
+      </c>
+      <c r="AH2" t="n">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -884,9 +890,15 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
+      <c r="AF3" t="n">
+        <v/>
+      </c>
+      <c r="AG3" t="n">
+        <v/>
+      </c>
+      <c r="AH3" t="n">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1034,9 +1046,15 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr"/>
+      <c r="AF4" t="n">
+        <v/>
+      </c>
+      <c r="AG4" t="n">
+        <v/>
+      </c>
+      <c r="AH4" t="n">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1184,9 +1202,15 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr"/>
+      <c r="AF5" t="n">
+        <v/>
+      </c>
+      <c r="AG5" t="n">
+        <v/>
+      </c>
+      <c r="AH5" t="n">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1334,9 +1358,15 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr"/>
+      <c r="AF6" t="n">
+        <v/>
+      </c>
+      <c r="AG6" t="n">
+        <v/>
+      </c>
+      <c r="AH6" t="n">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1484,9 +1514,15 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr"/>
+      <c r="AF7" t="n">
+        <v/>
+      </c>
+      <c r="AG7" t="n">
+        <v/>
+      </c>
+      <c r="AH7" t="n">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1634,9 +1670,15 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF8" t="inlineStr"/>
-      <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="inlineStr"/>
+      <c r="AF8" t="n">
+        <v/>
+      </c>
+      <c r="AG8" t="n">
+        <v/>
+      </c>
+      <c r="AH8" t="n">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1784,9 +1826,15 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF9" t="inlineStr"/>
-      <c r="AG9" t="inlineStr"/>
-      <c r="AH9" t="inlineStr"/>
+      <c r="AF9" t="n">
+        <v/>
+      </c>
+      <c r="AG9" t="n">
+        <v/>
+      </c>
+      <c r="AH9" t="n">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1934,9 +1982,15 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF10" t="inlineStr"/>
-      <c r="AG10" t="inlineStr"/>
-      <c r="AH10" t="inlineStr"/>
+      <c r="AF10" t="n">
+        <v/>
+      </c>
+      <c r="AG10" t="n">
+        <v/>
+      </c>
+      <c r="AH10" t="n">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2084,9 +2138,15 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF11" t="inlineStr"/>
-      <c r="AG11" t="inlineStr"/>
-      <c r="AH11" t="inlineStr"/>
+      <c r="AF11" t="n">
+        <v/>
+      </c>
+      <c r="AG11" t="n">
+        <v/>
+      </c>
+      <c r="AH11" t="n">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2234,9 +2294,15 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF12" t="inlineStr"/>
-      <c r="AG12" t="inlineStr"/>
-      <c r="AH12" t="inlineStr"/>
+      <c r="AF12" t="n">
+        <v/>
+      </c>
+      <c r="AG12" t="n">
+        <v/>
+      </c>
+      <c r="AH12" t="n">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2384,9 +2450,15 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF13" t="inlineStr"/>
-      <c r="AG13" t="inlineStr"/>
-      <c r="AH13" t="inlineStr"/>
+      <c r="AF13" t="n">
+        <v/>
+      </c>
+      <c r="AG13" t="n">
+        <v/>
+      </c>
+      <c r="AH13" t="n">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2534,9 +2606,15 @@
           <t>MVP-2a3 正常配平样例</t>
         </is>
       </c>
-      <c r="AF14" t="inlineStr"/>
-      <c r="AG14" t="inlineStr"/>
-      <c r="AH14" t="inlineStr"/>
+      <c r="AF14" t="n">
+        <v/>
+      </c>
+      <c r="AG14" t="n">
+        <v/>
+      </c>
+      <c r="AH14" t="n">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">

</xml_diff>

<commit_message>
chore: baseline deterministic xlsx fixtures
</commit_message>
<xml_diff>
--- a/mock_data/mvp2a3_core.xlsx
+++ b/mock_data/mvp2a3_core.xlsx
@@ -734,15 +734,9 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF2" t="n">
-        <v/>
-      </c>
-      <c r="AG2" t="n">
-        <v/>
-      </c>
-      <c r="AH2" t="n">
-        <v/>
-      </c>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -890,15 +884,9 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF3" t="n">
-        <v/>
-      </c>
-      <c r="AG3" t="n">
-        <v/>
-      </c>
-      <c r="AH3" t="n">
-        <v/>
-      </c>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1046,15 +1034,9 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF4" t="n">
-        <v/>
-      </c>
-      <c r="AG4" t="n">
-        <v/>
-      </c>
-      <c r="AH4" t="n">
-        <v/>
-      </c>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1202,15 +1184,9 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF5" t="n">
-        <v/>
-      </c>
-      <c r="AG5" t="n">
-        <v/>
-      </c>
-      <c r="AH5" t="n">
-        <v/>
-      </c>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1358,15 +1334,9 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF6" t="n">
-        <v/>
-      </c>
-      <c r="AG6" t="n">
-        <v/>
-      </c>
-      <c r="AH6" t="n">
-        <v/>
-      </c>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1514,15 +1484,9 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF7" t="n">
-        <v/>
-      </c>
-      <c r="AG7" t="n">
-        <v/>
-      </c>
-      <c r="AH7" t="n">
-        <v/>
-      </c>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1670,15 +1634,9 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF8" t="n">
-        <v/>
-      </c>
-      <c r="AG8" t="n">
-        <v/>
-      </c>
-      <c r="AH8" t="n">
-        <v/>
-      </c>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1826,15 +1784,9 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF9" t="n">
-        <v/>
-      </c>
-      <c r="AG9" t="n">
-        <v/>
-      </c>
-      <c r="AH9" t="n">
-        <v/>
-      </c>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1982,15 +1934,9 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF10" t="n">
-        <v/>
-      </c>
-      <c r="AG10" t="n">
-        <v/>
-      </c>
-      <c r="AH10" t="n">
-        <v/>
-      </c>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2138,15 +2084,9 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF11" t="n">
-        <v/>
-      </c>
-      <c r="AG11" t="n">
-        <v/>
-      </c>
-      <c r="AH11" t="n">
-        <v/>
-      </c>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2294,15 +2234,9 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF12" t="n">
-        <v/>
-      </c>
-      <c r="AG12" t="n">
-        <v/>
-      </c>
-      <c r="AH12" t="n">
-        <v/>
-      </c>
+      <c r="AF12" t="inlineStr"/>
+      <c r="AG12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2450,15 +2384,9 @@
           <t>清算批次正常自动平账样例</t>
         </is>
       </c>
-      <c r="AF13" t="n">
-        <v/>
-      </c>
-      <c r="AG13" t="n">
-        <v/>
-      </c>
-      <c r="AH13" t="n">
-        <v/>
-      </c>
+      <c r="AF13" t="inlineStr"/>
+      <c r="AG13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2606,15 +2534,9 @@
           <t>MVP-2a3 正常配平样例</t>
         </is>
       </c>
-      <c r="AF14" t="n">
-        <v/>
-      </c>
-      <c r="AG14" t="n">
-        <v/>
-      </c>
-      <c r="AH14" t="n">
-        <v/>
-      </c>
+      <c r="AF14" t="inlineStr"/>
+      <c r="AG14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">

</xml_diff>